<commit_message>
Ajuste Olimpica sum de importes de Facturas en Olimica Colombia
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_olimpica.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_olimpica.xlsx
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -786,7 +786,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>28/11/2025</t>
+          <t>02/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1254,16 +1254,16 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>PMP1286466</t>
+          <t>PMP1286467</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>640693961.84</v>
+        <v>137894507.16</v>
       </c>
       <c r="F33" s="10" t="inlineStr"/>
       <c r="G33" s="10" t="inlineStr"/>
       <c r="H33" s="6" t="n">
-        <v>640693961.84</v>
+        <v>137894507.16</v>
       </c>
       <c r="I33" s="11" t="inlineStr"/>
     </row>
@@ -1275,16 +1275,16 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>PMP1286467</t>
+          <t>PMP1291552</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>137894507.16</v>
+        <v>4175700</v>
       </c>
       <c r="F34" s="10" t="inlineStr"/>
       <c r="G34" s="10" t="inlineStr"/>
       <c r="H34" s="6" t="n">
-        <v>137894507.16</v>
+        <v>4175700</v>
       </c>
       <c r="I34" s="11" t="inlineStr"/>
     </row>
@@ -1296,16 +1296,16 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>PMP1291552</t>
+          <t>PMP1291553</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>4175700</v>
+        <v>41784946.6</v>
       </c>
       <c r="F35" s="10" t="inlineStr"/>
       <c r="G35" s="10" t="inlineStr"/>
       <c r="H35" s="6" t="n">
-        <v>4175700</v>
+        <v>41784946.6</v>
       </c>
       <c r="I35" s="11" t="inlineStr"/>
     </row>
@@ -1317,16 +1317,16 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>PMP1291553</t>
+          <t>PMP1291554</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>41784946.6</v>
+        <v>1230911.12</v>
       </c>
       <c r="F36" s="10" t="inlineStr"/>
       <c r="G36" s="10" t="inlineStr"/>
       <c r="H36" s="6" t="n">
-        <v>41784946.6</v>
+        <v>1230911.12</v>
       </c>
       <c r="I36" s="11" t="inlineStr"/>
     </row>
@@ -1338,16 +1338,16 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>PMP1291554</t>
+          <t>PMP1291555</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>1230911.12</v>
+        <v>347975</v>
       </c>
       <c r="F37" s="10" t="inlineStr"/>
       <c r="G37" s="10" t="inlineStr"/>
       <c r="H37" s="6" t="n">
-        <v>1230911.12</v>
+        <v>347975</v>
       </c>
       <c r="I37" s="11" t="inlineStr"/>
     </row>
@@ -1359,16 +1359,16 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>PMP1291555</t>
+          <t>PMP1291556</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>347975</v>
+        <v>47200684.8</v>
       </c>
       <c r="F38" s="10" t="inlineStr"/>
       <c r="G38" s="10" t="inlineStr"/>
       <c r="H38" s="6" t="n">
-        <v>347975</v>
+        <v>47200684.8</v>
       </c>
       <c r="I38" s="11" t="inlineStr"/>
     </row>
@@ -1380,16 +1380,16 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>PMP1291556</t>
+          <t>PMP1291557</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>47200684.8</v>
+        <v>173988</v>
       </c>
       <c r="F39" s="10" t="inlineStr"/>
       <c r="G39" s="10" t="inlineStr"/>
       <c r="H39" s="6" t="n">
-        <v>47200684.8</v>
+        <v>173988</v>
       </c>
       <c r="I39" s="11" t="inlineStr"/>
     </row>
@@ -1401,16 +1401,16 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>PMP1291557</t>
+          <t>PMP1291558</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>173988</v>
+        <v>554871.24</v>
       </c>
       <c r="F40" s="10" t="inlineStr"/>
       <c r="G40" s="10" t="inlineStr"/>
       <c r="H40" s="6" t="n">
-        <v>173988</v>
+        <v>554871.24</v>
       </c>
       <c r="I40" s="11" t="inlineStr"/>
     </row>
@@ -1422,16 +1422,16 @@
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>PMP1291558</t>
+          <t>PMP1291559</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>554871.24</v>
+        <v>7395026.5</v>
       </c>
       <c r="F41" s="10" t="inlineStr"/>
       <c r="G41" s="10" t="inlineStr"/>
       <c r="H41" s="6" t="n">
-        <v>554871.24</v>
+        <v>7395026.5</v>
       </c>
       <c r="I41" s="11" t="inlineStr"/>
     </row>
@@ -1443,16 +1443,16 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>PMP1291559</t>
+          <t>PMP1291560</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>7395026.5</v>
+        <v>62932310.75</v>
       </c>
       <c r="F42" s="10" t="inlineStr"/>
       <c r="G42" s="10" t="inlineStr"/>
       <c r="H42" s="6" t="n">
-        <v>7395026.5</v>
+        <v>62932310.75</v>
       </c>
       <c r="I42" s="11" t="inlineStr"/>
     </row>
@@ -1464,16 +1464,16 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>PMP1291560</t>
+          <t>PMP1291561</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>62932310.75</v>
+        <v>43153234.4</v>
       </c>
       <c r="F43" s="10" t="inlineStr"/>
       <c r="G43" s="10" t="inlineStr"/>
       <c r="H43" s="6" t="n">
-        <v>62932310.75</v>
+        <v>43153234.4</v>
       </c>
       <c r="I43" s="11" t="inlineStr"/>
     </row>
@@ -1485,16 +1485,16 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1291562</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>43153234.4</v>
+        <v>7043898.34</v>
       </c>
       <c r="F44" s="10" t="inlineStr"/>
       <c r="G44" s="10" t="inlineStr"/>
       <c r="H44" s="6" t="n">
-        <v>43153234.4</v>
+        <v>7043898.34</v>
       </c>
       <c r="I44" s="11" t="inlineStr"/>
     </row>
@@ -1506,16 +1506,16 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1291563</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>43153234.4</v>
+        <v>82462889.81999999</v>
       </c>
       <c r="F45" s="10" t="inlineStr"/>
       <c r="G45" s="10" t="inlineStr"/>
       <c r="H45" s="6" t="n">
-        <v>43153234.4</v>
+        <v>82462889.81999999</v>
       </c>
       <c r="I45" s="11" t="inlineStr"/>
     </row>
@@ -1527,16 +1527,16 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>PMP1291562</t>
+          <t>PMP1291965</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>7043898.34</v>
+        <v>7349759</v>
       </c>
       <c r="F46" s="10" t="inlineStr"/>
       <c r="G46" s="10" t="inlineStr"/>
       <c r="H46" s="6" t="n">
-        <v>7043898.34</v>
+        <v>7349759</v>
       </c>
       <c r="I46" s="11" t="inlineStr"/>
     </row>
@@ -1548,16 +1548,16 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>PMP1291563</t>
+          <t>PMP1292294</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>82462889.81999999</v>
+        <v>3131775</v>
       </c>
       <c r="F47" s="10" t="inlineStr"/>
       <c r="G47" s="10" t="inlineStr"/>
       <c r="H47" s="6" t="n">
-        <v>82462889.81999999</v>
+        <v>3131775</v>
       </c>
       <c r="I47" s="11" t="inlineStr"/>
     </row>
@@ -1569,16 +1569,16 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>PMP1291965</t>
+          <t>PMP1292295</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>7349759</v>
+        <v>86994</v>
       </c>
       <c r="F48" s="10" t="inlineStr"/>
       <c r="G48" s="10" t="inlineStr"/>
       <c r="H48" s="6" t="n">
-        <v>7349759</v>
+        <v>86994</v>
       </c>
       <c r="I48" s="11" t="inlineStr"/>
     </row>
@@ -1590,16 +1590,16 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>PMP1292294</t>
+          <t>PMP1292296</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>3131775</v>
+        <v>13811678.4</v>
       </c>
       <c r="F49" s="10" t="inlineStr"/>
       <c r="G49" s="10" t="inlineStr"/>
       <c r="H49" s="6" t="n">
-        <v>3131775</v>
+        <v>13811678.4</v>
       </c>
       <c r="I49" s="11" t="inlineStr"/>
     </row>
@@ -1611,16 +1611,16 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>PMP1292295</t>
+          <t>PMP1292297</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>86994</v>
+        <v>32030709.54</v>
       </c>
       <c r="F50" s="10" t="inlineStr"/>
       <c r="G50" s="10" t="inlineStr"/>
       <c r="H50" s="6" t="n">
-        <v>86994</v>
+        <v>32030709.54</v>
       </c>
       <c r="I50" s="11" t="inlineStr"/>
     </row>
@@ -1632,16 +1632,16 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>PMP1292296</t>
+          <t>PMP1292298</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>13811678.4</v>
+        <v>34758234.75</v>
       </c>
       <c r="F51" s="10" t="inlineStr"/>
       <c r="G51" s="10" t="inlineStr"/>
       <c r="H51" s="6" t="n">
-        <v>13811678.4</v>
+        <v>34758234.75</v>
       </c>
       <c r="I51" s="11" t="inlineStr"/>
     </row>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>PMP1292297</t>
+          <t>PMP1292309</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>32030709.54</v>
+        <v>20376764.8</v>
       </c>
       <c r="F52" s="10" t="inlineStr"/>
       <c r="G52" s="10" t="inlineStr"/>
       <c r="H52" s="6" t="n">
-        <v>32030709.54</v>
+        <v>20376764.8</v>
       </c>
       <c r="I52" s="11" t="inlineStr"/>
     </row>
@@ -1674,16 +1674,16 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>PMP1292298</t>
+          <t>PMP1292593</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>34758234.75</v>
+        <v>3131775</v>
       </c>
       <c r="F53" s="10" t="inlineStr"/>
       <c r="G53" s="10" t="inlineStr"/>
       <c r="H53" s="6" t="n">
-        <v>34758234.75</v>
+        <v>3131775</v>
       </c>
       <c r="I53" s="11" t="inlineStr"/>
     </row>
@@ -1695,16 +1695,16 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>PMP1292309</t>
+          <t>PMP1292594</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>20376764.8</v>
+        <v>30380459.6</v>
       </c>
       <c r="F54" s="10" t="inlineStr"/>
       <c r="G54" s="10" t="inlineStr"/>
       <c r="H54" s="6" t="n">
-        <v>20376764.8</v>
+        <v>30380459.6</v>
       </c>
       <c r="I54" s="11" t="inlineStr"/>
     </row>
@@ -1716,16 +1716,16 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>PMP1292593</t>
+          <t>PMP1292652</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>3131775</v>
+        <v>30145687</v>
       </c>
       <c r="F55" s="10" t="inlineStr"/>
       <c r="G55" s="10" t="inlineStr"/>
       <c r="H55" s="6" t="n">
-        <v>3131775</v>
+        <v>30145687</v>
       </c>
       <c r="I55" s="11" t="inlineStr"/>
     </row>
@@ -1737,16 +1737,16 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>PMP1292594</t>
+          <t>PMP1292653</t>
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>30380459.6</v>
+        <v>27925238.47</v>
       </c>
       <c r="F56" s="10" t="inlineStr"/>
       <c r="G56" s="10" t="inlineStr"/>
       <c r="H56" s="6" t="n">
-        <v>30380459.6</v>
+        <v>27925238.47</v>
       </c>
       <c r="I56" s="11" t="inlineStr"/>
     </row>
@@ -1758,16 +1758,16 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>PMP1292652</t>
+          <t>PMP1292654</t>
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>30145687</v>
+        <v>46242233.5</v>
       </c>
       <c r="F57" s="10" t="inlineStr"/>
       <c r="G57" s="10" t="inlineStr"/>
       <c r="H57" s="6" t="n">
-        <v>30145687</v>
+        <v>46242233.5</v>
       </c>
       <c r="I57" s="11" t="inlineStr"/>
     </row>
@@ -1779,16 +1779,16 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>PMP1292653</t>
+          <t>PMP1292704</t>
         </is>
       </c>
       <c r="E58" s="6" t="n">
-        <v>27925238.47</v>
+        <v>4192184.8</v>
       </c>
       <c r="F58" s="10" t="inlineStr"/>
       <c r="G58" s="10" t="inlineStr"/>
       <c r="H58" s="6" t="n">
-        <v>27925238.47</v>
+        <v>4192184.8</v>
       </c>
       <c r="I58" s="11" t="inlineStr"/>
     </row>
@@ -1800,16 +1800,16 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>PMP1292654</t>
+          <t>PMP1292712</t>
         </is>
       </c>
       <c r="E59" s="6" t="n">
-        <v>46242233.5</v>
+        <v>16403804</v>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
       <c r="G59" s="10" t="inlineStr"/>
       <c r="H59" s="6" t="n">
-        <v>46242233.5</v>
+        <v>16403804</v>
       </c>
       <c r="I59" s="11" t="inlineStr"/>
     </row>
@@ -1821,16 +1821,16 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>PMP1292704</t>
+          <t>PMP1292713</t>
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>4192184.8</v>
+        <v>31007952.84</v>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
       <c r="G60" s="10" t="inlineStr"/>
       <c r="H60" s="6" t="n">
-        <v>4192184.8</v>
+        <v>31007952.84</v>
       </c>
       <c r="I60" s="11" t="inlineStr"/>
     </row>
@@ -1842,60 +1842,84 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>PMP1292712</t>
+          <t>PMP1292714</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>16403804</v>
+        <v>32461435</v>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
       <c r="G61" s="10" t="inlineStr"/>
       <c r="H61" s="6" t="n">
-        <v>16403804</v>
+        <v>32461435</v>
       </c>
       <c r="I61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>PMP1292713</t>
+          <t>4636412647</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>31007952.84</v>
-      </c>
-      <c r="F62" s="10" t="inlineStr"/>
-      <c r="G62" s="10" t="inlineStr"/>
+        <v>-16320</v>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>AVERIA</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
       <c r="H62" s="6" t="n">
-        <v>31007952.84</v>
-      </c>
-      <c r="I62" s="11" t="inlineStr"/>
+        <v>-16320</v>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>AVERIA 4636412647</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>PMP1292714</t>
+          <t>0085501420</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>32461435</v>
-      </c>
-      <c r="F63" s="10" t="inlineStr"/>
-      <c r="G63" s="10" t="inlineStr"/>
+        <v>-11077235</v>
+      </c>
+      <c r="F63" s="10" t="inlineStr">
+        <is>
+          <t>DESCUENTO</t>
+        </is>
+      </c>
+      <c r="G63" s="10" t="inlineStr">
+        <is>
+          <t>987</t>
+        </is>
+      </c>
       <c r="H63" s="6" t="n">
-        <v>32461435</v>
-      </c>
-      <c r="I63" s="11" t="inlineStr"/>
+        <v>-11077235</v>
+      </c>
+      <c r="I63" s="11" t="inlineStr">
+        <is>
+          <t>DESCUENTO 0085501420</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="C64" s="10" t="inlineStr">
@@ -1905,28 +1929,28 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>4636412647</t>
+          <t>9801673296</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>-16320</v>
+        <v>-116500000</v>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>AVERIA</t>
+          <t>FACT PROVEEDOR</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H64" s="6" t="n">
-        <v>-16320</v>
+        <v>-116500000</v>
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 4636412647</t>
+          <t>FACT PROVEEDOR 9801673296</t>
         </is>
       </c>
     </row>
@@ -1938,94 +1962,94 @@
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>0085501420</t>
+          <t>9801673633</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>-11077235</v>
+        <v>-296234085</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO</t>
+          <t>FACT PROVEEDOR</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H65" s="6" t="n">
-        <v>-11077235</v>
+        <v>-296234085</v>
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO 0085501420</t>
+          <t>FACT PROVEEDOR 9801673633</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>9801673296</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>-116500000</v>
+        <v>-70.07999997888692</v>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H66" s="6" t="n">
-        <v>-116500000</v>
+        <v>-70.07999997888692</v>
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR 9801673296</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>9801673633</t>
+          <t>PMP1286466</t>
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>-296234085</v>
+        <v>4384856.159999967</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G67" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H67" s="6" t="n">
-        <v>-296234085</v>
+        <v>4384856.159999967</v>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR 9801673633</t>
+          <t>Myr Vlr Pagado PMP1286466</t>
         </is>
       </c>
     </row>
@@ -2037,94 +2061,94 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>PMP1291561</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>-81.3200000107754</v>
+        <v>869392.6000000015</v>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H68" s="6" t="n">
-        <v>-81.3200000107754</v>
+        <v>869392.6000000015</v>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Myr Vlr Pagado PMP1291561</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>PMP1286466</t>
+          <t>PMP1286182</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>-636309101.84</v>
+        <v>-232158</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G69" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H69" s="6" t="n">
-        <v>-636309101.84</v>
+        <v>-232158</v>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1286466</t>
+          <t>RECHAZO PMP1286182</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1286191</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>-42283834.4</v>
+        <v>-474381</v>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H70" s="6" t="n">
-        <v>-42283834.4</v>
+        <v>-474381</v>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>Menor Vlr Pagado PMP1291561</t>
+          <t>RECHAZO PMP1286191</t>
         </is>
       </c>
     </row>
@@ -2136,11 +2160,11 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>PMP1286182</t>
+          <t>PMP1286466</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>-232158</v>
+        <v>-4623481</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -2153,11 +2177,11 @@
         </is>
       </c>
       <c r="H71" s="6" t="n">
-        <v>-232158</v>
+        <v>-4623481</v>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286182</t>
+          <t>RECHAZO PMP1286466</t>
         </is>
       </c>
     </row>
@@ -2169,11 +2193,11 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>PMP1286191</t>
+          <t>PMP1291558</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>-474381</v>
+        <v>-7</v>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
@@ -2186,11 +2210,11 @@
         </is>
       </c>
       <c r="H72" s="6" t="n">
-        <v>-474381</v>
+        <v>-7</v>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286191</t>
+          <t>RECHAZO PMP1291558</t>
         </is>
       </c>
     </row>
@@ -2202,11 +2226,11 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>PMP1286466</t>
+          <t>PMP1291559</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>-4623481</v>
+        <v>-94939</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -2219,11 +2243,11 @@
         </is>
       </c>
       <c r="H73" s="6" t="n">
-        <v>-4623481</v>
+        <v>-94939</v>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286466</t>
+          <t>RECHAZO PMP1291559</t>
         </is>
       </c>
     </row>
@@ -2235,11 +2259,11 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>PMP1291558</t>
+          <t>PMP1291560</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>-7</v>
+        <v>-1101</v>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
@@ -2252,11 +2276,11 @@
         </is>
       </c>
       <c r="H74" s="6" t="n">
-        <v>-7</v>
+        <v>-1101</v>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291558</t>
+          <t>RECHAZO PMP1291560</t>
         </is>
       </c>
     </row>
@@ -2268,11 +2292,11 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>PMP1291559</t>
+          <t>PMP1291561</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>-94939</v>
+        <v>-869290</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -2285,11 +2309,11 @@
         </is>
       </c>
       <c r="H75" s="6" t="n">
-        <v>-94939</v>
+        <v>-869290</v>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291559</t>
+          <t>RECHAZO PMP1291561</t>
         </is>
       </c>
     </row>
@@ -2301,11 +2325,11 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>PMP1291560</t>
+          <t>PMP1291563</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>-1101</v>
+        <v>-8705</v>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
@@ -2318,11 +2342,11 @@
         </is>
       </c>
       <c r="H76" s="6" t="n">
-        <v>-1101</v>
+        <v>-8705</v>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291560</t>
+          <t>RECHAZO PMP1291563</t>
         </is>
       </c>
     </row>
@@ -2334,11 +2358,11 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1291965</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>-869290</v>
+        <v>-153246</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -2351,11 +2375,11 @@
         </is>
       </c>
       <c r="H77" s="6" t="n">
-        <v>-869290</v>
+        <v>-153246</v>
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291561</t>
+          <t>RECHAZO PMP1291965</t>
         </is>
       </c>
     </row>
@@ -2367,11 +2391,11 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1291563</t>
+          <t>PMP1292298</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>-8705</v>
+        <v>-608</v>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
@@ -2384,11 +2408,11 @@
         </is>
       </c>
       <c r="H78" s="6" t="n">
-        <v>-8705</v>
+        <v>-608</v>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291563</t>
+          <t>RECHAZO PMP1292298</t>
         </is>
       </c>
     </row>
@@ -2400,11 +2424,11 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>PMP1291965</t>
+          <t>PMP1292652</t>
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>-153246</v>
+        <v>-143</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -2417,11 +2441,11 @@
         </is>
       </c>
       <c r="H79" s="6" t="n">
-        <v>-153246</v>
+        <v>-143</v>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291965</t>
+          <t>RECHAZO PMP1292652</t>
         </is>
       </c>
     </row>
@@ -2433,11 +2457,11 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>PMP1292298</t>
+          <t>PMP1292654</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>-608</v>
+        <v>-808</v>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
@@ -2450,11 +2474,11 @@
         </is>
       </c>
       <c r="H80" s="6" t="n">
-        <v>-608</v>
+        <v>-808</v>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292298</t>
+          <t>RECHAZO PMP1292654</t>
         </is>
       </c>
     </row>
@@ -2466,11 +2490,11 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>PMP1292652</t>
+          <t>PMP1292712</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>-143</v>
+        <v>-68</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -2483,11 +2507,11 @@
         </is>
       </c>
       <c r="H81" s="6" t="n">
-        <v>-143</v>
+        <v>-68</v>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292652</t>
+          <t>RECHAZO PMP1292712</t>
         </is>
       </c>
     </row>
@@ -2499,11 +2523,11 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>PMP1292654</t>
+          <t>PMP1292713</t>
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>-808</v>
+        <v>-9</v>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
@@ -2516,11 +2540,11 @@
         </is>
       </c>
       <c r="H82" s="6" t="n">
-        <v>-808</v>
+        <v>-9</v>
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292654</t>
+          <t>RECHAZO PMP1292713</t>
         </is>
       </c>
     </row>
@@ -2532,11 +2556,11 @@
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>PMP1292712</t>
+          <t>PMP1292714</t>
         </is>
       </c>
       <c r="E83" s="6" t="n">
-        <v>-68</v>
+        <v>-567</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -2549,75 +2573,9 @@
         </is>
       </c>
       <c r="H83" s="6" t="n">
-        <v>-68</v>
+        <v>-567</v>
       </c>
       <c r="I83" s="11" t="inlineStr">
-        <is>
-          <t>RECHAZO PMP1292712</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Cliente</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="inlineStr">
-        <is>
-          <t>PMP1292713</t>
-        </is>
-      </c>
-      <c r="E84" s="6" t="n">
-        <v>-9</v>
-      </c>
-      <c r="F84" s="10" t="inlineStr">
-        <is>
-          <t>RECHAZO</t>
-        </is>
-      </c>
-      <c r="G84" s="10" t="inlineStr">
-        <is>
-          <t>551</t>
-        </is>
-      </c>
-      <c r="H84" s="6" t="n">
-        <v>-9</v>
-      </c>
-      <c r="I84" s="11" t="inlineStr">
-        <is>
-          <t>RECHAZO PMP1292713</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Cliente</t>
-        </is>
-      </c>
-      <c r="D85" s="10" t="inlineStr">
-        <is>
-          <t>PMP1292714</t>
-        </is>
-      </c>
-      <c r="E85" s="6" t="n">
-        <v>-567</v>
-      </c>
-      <c r="F85" s="10" t="inlineStr">
-        <is>
-          <t>RECHAZO</t>
-        </is>
-      </c>
-      <c r="G85" s="10" t="inlineStr">
-        <is>
-          <t>551</t>
-        </is>
-      </c>
-      <c r="H85" s="6" t="n">
-        <v>-567</v>
-      </c>
-      <c r="I85" s="11" t="inlineStr">
         <is>
           <t>RECHAZO PMP1292714</t>
         </is>

</xml_diff>

<commit_message>
Mejora de entorno de pruebas
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_olimpica.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_olimpica.xlsx
@@ -898,7 +898,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>02/12/2025</t>
+          <t>04/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1858,66 +1858,66 @@
     <row r="62">
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>4636412647</t>
+          <t>PMP1286466</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>-16320</v>
+        <v>4384856.159999967</v>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>AVERIA</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H62" s="6" t="n">
-        <v>-16320</v>
+        <v>4384856.159999967</v>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 4636412647</t>
+          <t>Myr Vlr Pagado PMP1286466</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>0085501420</t>
+          <t>PMP1291561</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>-11077235</v>
+        <v>869392.6000000015</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO</t>
+          <t>Myr Vlr Pagado</t>
         </is>
       </c>
       <c r="G63" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>388</t>
         </is>
       </c>
       <c r="H63" s="6" t="n">
-        <v>-11077235</v>
+        <v>869392.6000000015</v>
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO 0085501420</t>
+          <t>Myr Vlr Pagado PMP1291561</t>
         </is>
       </c>
     </row>
@@ -1929,28 +1929,28 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>9801673296</t>
+          <t>4636412647</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>-116500000</v>
+        <v>-16320</v>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>AVERIA</t>
         </is>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>522</t>
         </is>
       </c>
       <c r="H64" s="6" t="n">
-        <v>-116500000</v>
+        <v>-16320</v>
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR 9801673296</t>
+          <t>AVERIA 4636412647</t>
         </is>
       </c>
     </row>
@@ -1962,68 +1962,68 @@
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>9801673633</t>
+          <t>PMP1286182</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>-296234085</v>
+        <v>-232158</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H65" s="6" t="n">
-        <v>-296234085</v>
+        <v>-232158</v>
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR 9801673633</t>
+          <t>RECHAZO PMP1286182</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>PMP1286191</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>-70.07999997888692</v>
+        <v>-474381</v>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H66" s="6" t="n">
-        <v>-70.07999997888692</v>
+        <v>-474381</v>
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>RECHAZO PMP1286191</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -2032,57 +2032,57 @@
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>4384856.159999967</v>
+        <v>-4623481</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G67" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H67" s="6" t="n">
-        <v>4384856.159999967</v>
+        <v>-4623481</v>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1286466</t>
+          <t>RECHAZO PMP1286466</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuentos Cliente</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1291558</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>869392.6000000015</v>
+        <v>-7</v>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado</t>
+          <t>RECHAZO</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>551</t>
         </is>
       </c>
       <c r="H68" s="6" t="n">
-        <v>869392.6000000015</v>
+        <v>-7</v>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>Myr Vlr Pagado PMP1291561</t>
+          <t>RECHAZO PMP1291558</t>
         </is>
       </c>
     </row>
@@ -2094,11 +2094,11 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>PMP1286182</t>
+          <t>PMP1291559</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>-232158</v>
+        <v>-94939</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -2111,11 +2111,11 @@
         </is>
       </c>
       <c r="H69" s="6" t="n">
-        <v>-232158</v>
+        <v>-94939</v>
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286182</t>
+          <t>RECHAZO PMP1291559</t>
         </is>
       </c>
     </row>
@@ -2127,11 +2127,11 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>PMP1286191</t>
+          <t>PMP1291560</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>-474381</v>
+        <v>-1101</v>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
@@ -2144,11 +2144,11 @@
         </is>
       </c>
       <c r="H70" s="6" t="n">
-        <v>-474381</v>
+        <v>-1101</v>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286191</t>
+          <t>RECHAZO PMP1291560</t>
         </is>
       </c>
     </row>
@@ -2160,11 +2160,11 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>PMP1286466</t>
+          <t>PMP1291561</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>-4623481</v>
+        <v>-869290</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -2177,11 +2177,11 @@
         </is>
       </c>
       <c r="H71" s="6" t="n">
-        <v>-4623481</v>
+        <v>-869290</v>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1286466</t>
+          <t>RECHAZO PMP1291561</t>
         </is>
       </c>
     </row>
@@ -2193,11 +2193,11 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>PMP1291558</t>
+          <t>PMP1291563</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>-7</v>
+        <v>-8705</v>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
@@ -2210,11 +2210,11 @@
         </is>
       </c>
       <c r="H72" s="6" t="n">
-        <v>-7</v>
+        <v>-8705</v>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291558</t>
+          <t>RECHAZO PMP1291563</t>
         </is>
       </c>
     </row>
@@ -2226,11 +2226,11 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>PMP1291559</t>
+          <t>PMP1291965</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>-94939</v>
+        <v>-153246</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -2243,11 +2243,11 @@
         </is>
       </c>
       <c r="H73" s="6" t="n">
-        <v>-94939</v>
+        <v>-153246</v>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291559</t>
+          <t>RECHAZO PMP1291965</t>
         </is>
       </c>
     </row>
@@ -2259,11 +2259,11 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>PMP1291560</t>
+          <t>PMP1292298</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>-1101</v>
+        <v>-608</v>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
@@ -2276,11 +2276,11 @@
         </is>
       </c>
       <c r="H74" s="6" t="n">
-        <v>-1101</v>
+        <v>-608</v>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291560</t>
+          <t>RECHAZO PMP1292298</t>
         </is>
       </c>
     </row>
@@ -2292,11 +2292,11 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>PMP1291561</t>
+          <t>PMP1292652</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>-869290</v>
+        <v>-143</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -2309,11 +2309,11 @@
         </is>
       </c>
       <c r="H75" s="6" t="n">
-        <v>-869290</v>
+        <v>-143</v>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291561</t>
+          <t>RECHAZO PMP1292652</t>
         </is>
       </c>
     </row>
@@ -2325,11 +2325,11 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>PMP1291563</t>
+          <t>PMP1292654</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>-8705</v>
+        <v>-808</v>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
@@ -2342,11 +2342,11 @@
         </is>
       </c>
       <c r="H76" s="6" t="n">
-        <v>-8705</v>
+        <v>-808</v>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291563</t>
+          <t>RECHAZO PMP1292654</t>
         </is>
       </c>
     </row>
@@ -2358,11 +2358,11 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>PMP1291965</t>
+          <t>PMP1292712</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>-153246</v>
+        <v>-68</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -2375,11 +2375,11 @@
         </is>
       </c>
       <c r="H77" s="6" t="n">
-        <v>-153246</v>
+        <v>-68</v>
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1291965</t>
+          <t>RECHAZO PMP1292712</t>
         </is>
       </c>
     </row>
@@ -2391,11 +2391,11 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1292298</t>
+          <t>PMP1292713</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>-608</v>
+        <v>-9</v>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
@@ -2408,11 +2408,11 @@
         </is>
       </c>
       <c r="H78" s="6" t="n">
-        <v>-608</v>
+        <v>-9</v>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292298</t>
+          <t>RECHAZO PMP1292713</t>
         </is>
       </c>
     </row>
@@ -2424,11 +2424,11 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>PMP1292652</t>
+          <t>PMP1292714</t>
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>-143</v>
+        <v>-567</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -2441,11 +2441,11 @@
         </is>
       </c>
       <c r="H79" s="6" t="n">
-        <v>-143</v>
+        <v>-567</v>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292652</t>
+          <t>RECHAZO PMP1292714</t>
         </is>
       </c>
     </row>
@@ -2457,28 +2457,28 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>PMP1292654</t>
+          <t>0085501420</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>-808</v>
+        <v>-11077235</v>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>RECHAZO</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="G80" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H80" s="6" t="n">
-        <v>-808</v>
+        <v>-11077235</v>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292654</t>
+          <t>DESCUENTO 0085501420</t>
         </is>
       </c>
     </row>
@@ -2490,28 +2490,28 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>PMP1292712</t>
+          <t>9801673296</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>-68</v>
+        <v>-116500000</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>RECHAZO</t>
+          <t>FACT PROVEEDOR</t>
         </is>
       </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H81" s="6" t="n">
-        <v>-68</v>
+        <v>-116500000</v>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292712</t>
+          <t>FACT PROVEEDOR 9801673296</t>
         </is>
       </c>
     </row>
@@ -2523,61 +2523,61 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>PMP1292713</t>
+          <t>9801673633</t>
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>-9</v>
+        <v>-296234085</v>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>RECHAZO</t>
+          <t>FACT PROVEEDOR</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H82" s="6" t="n">
-        <v>-9</v>
+        <v>-296234085</v>
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292713</t>
+          <t>FACT PROVEEDOR 9801673633</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>PMP1292714</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E83" s="6" t="n">
-        <v>-567</v>
+        <v>-70.07999997888692</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>RECHAZO</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G83" s="10" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H83" s="6" t="n">
-        <v>-567</v>
+        <v>-70.07999997888692</v>
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>RECHAZO PMP1292714</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>

</xml_diff>